<commit_message>
Improve parsing: header-repeating table blocks, PDF tables, optional OCR
- split XLSX/CSV into row blocks that repeat the header, so every chunk is
  self-describing; cap at XLSX_MAX_ROWS with a warning instead of silently
  truncating
- extract PDF tables per page with pdfplumber when installed
  (PDF_TABLES_ENABLED); fall back to plain text if the dependency is missing
- OCR scanned pages with pdf2image + pytesseract when a page has too little
  text (OCR_ENABLED, off by default), tagging metadata.ocr
- keep metadata keys unchanged so no Milvus re-ingestion is required
- extend the Demo workbook with a 24-row Roster sheet to exercise splitting
- add tests/test_parsing.py (13 cases) and an xlsx header assertion to
  check_loaders.py; document the new settings in the guide and .env.example
- suite is now 300 tests, coverage 92%
</commit_message>
<xml_diff>
--- a/data/Demo/metrics.xlsx
+++ b/data/Demo/metrics.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -516,4 +517,520 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>employee_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>on_call_week</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Employee 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Employee 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Employee 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Employee 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Employee 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Employee 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Employee 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Employee 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Employee 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Employee 10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Employee 11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Employee 12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Employee 13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Employee 14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Employee 15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Employee 16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Employee 17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Employee 18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Employee 19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Employee 20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Employee 21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Employee 22</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Employee 23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Employee 24</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>